<commit_message>
Guru 99 Banking System update
</commit_message>
<xml_diff>
--- a/Guru 99/SRS GURU99.xlsx
+++ b/Guru 99/SRS GURU99.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Games\3mk\Manual Testing\Guru 99\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9353BD47-5DDD-4094-8A1E-5F0B0828168D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43828140-8CE4-47D0-9DE5-D818570188CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{46F18F15-F5BE-4E77-8066-124D7813421F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="285">
   <si>
     <t>Title</t>
   </si>
@@ -223,10 +223,6 @@
     <t>"000145"</t>
   </si>
   <si>
-    <t>1-Write test data in customer ID field 
-3-Click on "Submit" button</t>
-  </si>
-  <si>
     <t>System should accept Customer ID and preserve leading zeros (if system treats ID as string) OR clarify behavior with requirement owner</t>
   </si>
   <si>
@@ -324,9 +320,6 @@
     <t>Cairo</t>
   </si>
   <si>
-    <t>System accepts valid Address and allows proceeding to next step</t>
-  </si>
-  <si>
     <t>TC_NC_City_001</t>
   </si>
   <si>
@@ -349,9 +342,6 @@
   </si>
   <si>
     <t>Verify City with valid input</t>
-  </si>
-  <si>
-    <t>System accepts valid City and allows proceeding to next step</t>
   </si>
   <si>
     <t>1-Leave City field empty
@@ -406,9 +396,6 @@
 2-Click on "Submit" button</t>
   </si>
   <si>
-    <t>System accepts valid State input and allows proceeding to next step</t>
-  </si>
-  <si>
     <t>System should display error message "State is required"</t>
   </si>
   <si>
@@ -466,9 +453,6 @@
     <t>" 1234"</t>
   </si>
   <si>
-    <t>System accepts valid PIN input and allows proceeding to next step</t>
-  </si>
-  <si>
     <t>TC_NC_PIN_006</t>
   </si>
   <si>
@@ -522,9 +506,6 @@
     <t>Verify Telephone number with valid input</t>
   </si>
   <si>
-    <t>System accepts valid Telephone number input and allows proceeding to next step</t>
-  </si>
-  <si>
     <t>444@134#13$4%</t>
   </si>
   <si>
@@ -602,9 +583,6 @@
 2-Click on "Submit" button</t>
   </si>
   <si>
-    <t>System accepts valid Email input and allows proceeding to next step</t>
-  </si>
-  <si>
     <t>TC_NC_Email_005</t>
   </si>
   <si>
@@ -648,6 +626,309 @@
   </si>
   <si>
     <t>System should reject malicious input, prevent execution, and display generic validation error without exposing system details</t>
+  </si>
+  <si>
+    <t>Balance Enquiry</t>
+  </si>
+  <si>
+    <t>TC_BE_001</t>
+  </si>
+  <si>
+    <t>TC_BE_002</t>
+  </si>
+  <si>
+    <t>TC_BE_003</t>
+  </si>
+  <si>
+    <t>Verify Account number is required</t>
+  </si>
+  <si>
+    <t>Verify Account number can't accept characters</t>
+  </si>
+  <si>
+    <t>Verify Account number can't accept special characters</t>
+  </si>
+  <si>
+    <t>TC_BE_004</t>
+  </si>
+  <si>
+    <t>Verify Account number with valid input</t>
+  </si>
+  <si>
+    <t>1ab2cd3</t>
+  </si>
+  <si>
+    <t>1@3##h%</t>
+  </si>
+  <si>
+    <t>1-Leave Account number field empty
+2-Click on "Submit" button</t>
+  </si>
+  <si>
+    <t>1-Write test data in Account number field
+2-Click on "Submit" button</t>
+  </si>
+  <si>
+    <t>System should display error message "Account number is required"</t>
+  </si>
+  <si>
+    <t>Customized Statement Form</t>
+  </si>
+  <si>
+    <t>TC_CSF_AccNO_001</t>
+  </si>
+  <si>
+    <t>TC_CSF_AccNO_002</t>
+  </si>
+  <si>
+    <t>TC_CSF_AccNO_003</t>
+  </si>
+  <si>
+    <t>TC_CSF_AccNO_004</t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_001</t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_002</t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_003</t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_004</t>
+  </si>
+  <si>
+    <t>TC_BE_005</t>
+  </si>
+  <si>
+    <t>Verify Reset button</t>
+  </si>
+  <si>
+    <t>Account num=1234567</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-Write test data in Account number field
+2-Click on "Reset" button
+</t>
+  </si>
+  <si>
+    <t>TC_NC_State_006</t>
+  </si>
+  <si>
+    <t>Verify state with only spaces</t>
+  </si>
+  <si>
+    <t>"        "</t>
+  </si>
+  <si>
+    <t>System should validate input (Clarification required)</t>
+  </si>
+  <si>
+    <t>Verify Amount Lower Limit is required</t>
+  </si>
+  <si>
+    <t>Verify Amount Lower Limit can't accept special characters</t>
+  </si>
+  <si>
+    <t>Verify Amount Lower Limit can't accept characters</t>
+  </si>
+  <si>
+    <t>1$%j^@</t>
+  </si>
+  <si>
+    <t>1bc23</t>
+  </si>
+  <si>
+    <t>1-Leave Amount lower limit empty
+2-Click on "Submit" button</t>
+  </si>
+  <si>
+    <t>System should display error message "Amount lower limit is required"</t>
+  </si>
+  <si>
+    <t>1-Write test data in Amount lower limit field
+2-Click on "Submit" button</t>
+  </si>
+  <si>
+    <t>Verify Amount Lower limit</t>
+  </si>
+  <si>
+    <t>System should reject zero amount if minimum amount &gt; 0 OR accept if zero is allowed (Clarification Required)</t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_005</t>
+  </si>
+  <si>
+    <t>Verify negative amount in amount lower limit</t>
+  </si>
+  <si>
+    <t>System should reject negative amount if minimum amount &gt; 0 (Clarification Required)</t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_006</t>
+  </si>
+  <si>
+    <t>Verify Decimal amount in amount lower limit</t>
+  </si>
+  <si>
+    <t>System should validate amount (Clarification Required)</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_001</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_002</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_003</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_004</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_005</t>
+  </si>
+  <si>
+    <t>Verify Number of Transaction is required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Number of Transaction </t>
+  </si>
+  <si>
+    <t>TC_CSF_AMLL_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Amount lower limit with valid input </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Number of Transaction can't accept characters </t>
+  </si>
+  <si>
+    <t>Verify Number of Transaction  can't accept special characters</t>
+  </si>
+  <si>
+    <t>Verify negative amount in Number Of Transaction</t>
+  </si>
+  <si>
+    <t>Verify Decimal amount in Number Of Transaction</t>
+  </si>
+  <si>
+    <t>Verify Zero in Number Of Transaction</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_006</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_007</t>
+  </si>
+  <si>
+    <t>1@3$</t>
+  </si>
+  <si>
+    <t>1-Leave Number Of Transaction empty
+2-Click on "Submit" button</t>
+  </si>
+  <si>
+    <t>1-Write test data in Number Of Transaction field
+2-Click on "Submit" button</t>
+  </si>
+  <si>
+    <t>System should display error message "characters are not allowed"</t>
+  </si>
+  <si>
+    <t>System should validate input (Clarification Required)</t>
+  </si>
+  <si>
+    <t>System should display error message "Number Of Transaction is required"</t>
+  </si>
+  <si>
+    <t>TC_CSF_NOT_008</t>
+  </si>
+  <si>
+    <t>Account Number=1234567
+Amount Lower Limit=1
+Number Of Transaction=1</t>
+  </si>
+  <si>
+    <t>1-Write test data in Number Of Transaction field
+2-Click on "Reset" button</t>
+  </si>
+  <si>
+    <t>User is on "New Customer" page</t>
+  </si>
+  <si>
+    <t>User is on "Balance Enquiry" page</t>
+  </si>
+  <si>
+    <t>User is on "Customized Statement Form" page</t>
+  </si>
+  <si>
+    <t>User is on "New Account" page</t>
+  </si>
+  <si>
+    <t>TC_NC_Email_007</t>
+  </si>
+  <si>
+    <t>Verify invalid Email format (Missing User name)</t>
+  </si>
+  <si>
+    <t>@test.com</t>
+  </si>
+  <si>
+    <t>TC_NC_Email_008</t>
+  </si>
+  <si>
+    <t>TC_NC_Email_009</t>
+  </si>
+  <si>
+    <t>Verify invalid Email format (Missing TLD)</t>
+  </si>
+  <si>
+    <t>Verify invalid Email format (Double @)</t>
+  </si>
+  <si>
+    <t>test@test</t>
+  </si>
+  <si>
+    <t>test@@test.com</t>
+  </si>
+  <si>
+    <t>All input fields should be cleared and reset to default state</t>
+  </si>
+  <si>
+    <t>System accepts the valid Customer Name without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid Address without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid City without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid State input without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid PIN input without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid Telephone number without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid Email without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid Account number without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid Amount Lower Limit without validation error</t>
+  </si>
+  <si>
+    <t>System accepts the valid Number of Transactions without validation error</t>
+  </si>
+  <si>
+    <t>1-Write test data in customer ID field 
+2-Click on "Submit" button</t>
   </si>
 </sst>
 </file>
@@ -761,7 +1042,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -787,10 +1068,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1128,13 +1415,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{464BCA4F-0A8B-44B3-9B6B-32816FD63C1C}">
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
     <col min="2" max="2" width="17.88671875" style="6" customWidth="1"/>
     <col min="3" max="3" width="28.6640625" customWidth="1"/>
-    <col min="4" max="4" width="34.77734375" customWidth="1"/>
+    <col min="4" max="4" width="39.21875" customWidth="1"/>
     <col min="5" max="5" width="21.33203125" customWidth="1"/>
     <col min="6" max="6" width="18.77734375" customWidth="1"/>
     <col min="7" max="7" width="36.6640625" customWidth="1"/>
@@ -1181,7 +1468,9 @@
       <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="5"/>
+      <c r="D2" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E2" s="5" t="s">
         <v>53</v>
       </c>
@@ -1204,7 +1493,9 @@
       <c r="C3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="5"/>
+      <c r="D3" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E3" s="8" t="s">
         <v>52</v>
       </c>
@@ -1227,7 +1518,9 @@
       <c r="C4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="5"/>
+      <c r="D4" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1250,7 +1543,9 @@
       <c r="C5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="5"/>
+      <c r="D5" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E5" s="5">
         <v>1234</v>
       </c>
@@ -1271,9 +1566,11 @@
         <v>17</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="D6" s="5"/>
+        <v>167</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E6" s="5">
         <v>123</v>
       </c>
@@ -1296,7 +1593,9 @@
       <c r="C7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="5"/>
+      <c r="D7" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E7" s="5" t="s">
         <v>54</v>
       </c>
@@ -1319,7 +1618,9 @@
       <c r="C8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="5"/>
+      <c r="D8" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E8" s="8" t="s">
         <v>31</v>
       </c>
@@ -1327,7 +1628,7 @@
         <v>32</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -1342,7 +1643,9 @@
       <c r="C9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="5"/>
+      <c r="D9" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E9" s="5" t="s">
         <v>34</v>
       </c>
@@ -1365,7 +1668,9 @@
       <c r="C10" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="5"/>
+      <c r="D10" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
@@ -1373,7 +1678,7 @@
         <v>32</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -1388,7 +1693,9 @@
       <c r="C11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="5"/>
+      <c r="D11" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E11" s="5">
         <v>11223134455</v>
       </c>
@@ -1396,7 +1703,7 @@
         <v>32</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -1411,7 +1718,9 @@
       <c r="C12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="5"/>
+      <c r="D12" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E12" s="8" t="s">
         <v>51</v>
       </c>
@@ -1434,7 +1743,9 @@
       <c r="C13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="5"/>
+      <c r="D13" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E13" s="5">
         <v>415236589</v>
       </c>
@@ -1457,127 +1768,139 @@
       <c r="C14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="5"/>
+      <c r="D14" s="12" t="s">
+        <v>263</v>
+      </c>
       <c r="E14" s="5" t="s">
         <v>57</v>
       </c>
       <c r="F14" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
     <row r="15" spans="1:9" ht="55.8" thickBot="1">
       <c r="A15" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>61</v>
-      </c>
       <c r="C15" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="5"/>
+        <v>66</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E15" s="5" t="s">
         <v>53</v>
       </c>
       <c r="F15" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>69</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
     <row r="16" spans="1:9" ht="69.599999999999994" thickBot="1">
       <c r="A16" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
     <row r="17" spans="1:9" ht="69.599999999999994" thickBot="1">
       <c r="A17" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D17" s="5"/>
+        <v>72</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E17" s="5">
         <v>1232654</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
     <row r="18" spans="1:9" ht="69.599999999999994" thickBot="1">
       <c r="A18" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D18" s="5"/>
+        <v>73</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E18" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>77</v>
+        <v>274</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
     </row>
     <row r="19" spans="1:9" ht="69.599999999999994" thickBot="1">
       <c r="A19" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="D19" s="5"/>
+        <v>166</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E19" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>46</v>
@@ -1587,1203 +1910,1936 @@
     </row>
     <row r="20" spans="1:9" ht="69.599999999999994" thickBot="1">
       <c r="A20" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="D20" s="5"/>
+        <v>185</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E20" s="5" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
     </row>
     <row r="21" spans="1:9" ht="55.8" thickBot="1">
       <c r="A21" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D21" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E21" s="5" t="s">
         <v>53</v>
       </c>
       <c r="F21" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
     </row>
     <row r="22" spans="1:9" ht="55.8" thickBot="1">
       <c r="A22" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C22" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="5"/>
-      <c r="E22" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>85</v>
-      </c>
       <c r="G22" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
     </row>
     <row r="23" spans="1:9" ht="55.8" thickBot="1">
       <c r="A23" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="D23" s="5"/>
+        <v>165</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E23" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="1"/>
+      <c r="H23" s="5"/>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" ht="55.8" thickBot="1">
       <c r="A24" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>88</v>
+      <c r="D24" s="12" t="s">
+        <v>260</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="H24" s="1"/>
+        <v>275</v>
+      </c>
+      <c r="H24" s="5"/>
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="1:9" ht="55.8" thickBot="1">
       <c r="A25" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="D25" s="5"/>
+        <v>95</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E25" s="8" t="s">
         <v>53</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="H25" s="1"/>
+        <v>98</v>
+      </c>
+      <c r="H25" s="5"/>
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:9" ht="55.8" thickBot="1">
       <c r="A26" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D26" s="5"/>
+        <v>94</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E26" s="8" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H26" s="1"/>
+        <v>71</v>
+      </c>
+      <c r="H26" s="5"/>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" ht="55.8" thickBot="1">
       <c r="A27" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="5"/>
+        <v>164</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E27" s="8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H27" s="1"/>
+      <c r="H27" s="5"/>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" ht="54" thickBot="1">
       <c r="A28" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D28" s="5"/>
+        <v>102</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E28" s="8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="H28" s="1"/>
+        <v>103</v>
+      </c>
+      <c r="H28" s="5"/>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" ht="54" thickBot="1">
       <c r="A29" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="D29" s="5"/>
+        <v>96</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E29" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="H29" s="1"/>
+        <v>276</v>
+      </c>
+      <c r="H29" s="5"/>
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="54" thickBot="1">
       <c r="A30" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="D30" s="5"/>
+        <v>117</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E30" s="8" t="s">
         <v>53</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="H30" s="1"/>
+        <v>113</v>
+      </c>
+      <c r="H30" s="5"/>
       <c r="I30" s="2"/>
     </row>
     <row r="31" spans="1:9" ht="54" thickBot="1">
       <c r="A31" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D31" s="5"/>
+        <v>116</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E31" s="8" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H31" s="1"/>
+        <v>71</v>
+      </c>
+      <c r="H31" s="5"/>
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" ht="54" thickBot="1">
       <c r="A32" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="8" t="s">
-        <v>112</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>106</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="H32" s="5"/>
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" ht="54" thickBot="1">
       <c r="A33" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D33" s="5"/>
+        <v>163</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E33" s="8" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>46</v>
       </c>
+      <c r="H33" s="5"/>
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" ht="54" thickBot="1">
       <c r="A34" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D34" s="5"/>
+        <v>114</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E34" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>116</v>
-      </c>
+        <v>277</v>
+      </c>
+      <c r="H34" s="5"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" ht="54" thickBot="1">
       <c r="A35" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>122</v>
+        <v>215</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D35" s="5"/>
+        <v>216</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E35" s="8" t="s">
-        <v>53</v>
+        <v>217</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>131</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="H35" s="5"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" ht="54" thickBot="1">
       <c r="A36" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B36" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="D36" s="5"/>
+      <c r="D36" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E36" s="8" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>24</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="H36" s="5"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" ht="54" thickBot="1">
       <c r="A37" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>132</v>
-      </c>
       <c r="G37" s="4" t="s">
-        <v>72</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="H37" s="5"/>
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" ht="54" thickBot="1">
       <c r="A38" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="D38" s="5"/>
+        <v>124</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E38" s="8" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>46</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="H38" s="5"/>
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" ht="54" thickBot="1">
       <c r="A39" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D39" s="5"/>
-      <c r="E39" s="8">
-        <v>123456</v>
+        <v>162</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>130</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>135</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H39" s="5"/>
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" ht="54" thickBot="1">
       <c r="A40" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D40" s="5"/>
+        <v>133</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E40" s="8">
-        <v>12345</v>
+        <v>123456</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>151</v>
-      </c>
+        <v>278</v>
+      </c>
+      <c r="H40" s="5"/>
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" ht="54" thickBot="1">
       <c r="A41" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D41" s="5"/>
+        <v>134</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E41" s="8">
-        <v>1234567</v>
+        <v>12345</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>151</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="H41" s="5"/>
       <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" ht="54" thickBot="1">
       <c r="A42" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="D42" s="5"/>
-      <c r="E42" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E42" s="8">
+        <v>1234567</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="H42" s="5"/>
+      <c r="I42" s="1"/>
+    </row>
+    <row r="43" spans="1:9" ht="54" thickBot="1">
+      <c r="A43" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E43" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="1:9" ht="67.2" thickBot="1">
-      <c r="A43" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B43" s="5" t="s">
+      <c r="F43" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C43" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D43" s="5"/>
-      <c r="E43" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>150</v>
-      </c>
       <c r="G43" s="4" t="s">
-        <v>72</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="H43" s="5"/>
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" ht="67.2" thickBot="1">
       <c r="A44" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D44" s="5"/>
+        <v>141</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E44" s="8" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>24</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="H44" s="5"/>
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" ht="67.2" thickBot="1">
       <c r="A45" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B45" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="C45" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D45" s="5"/>
+      <c r="D45" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E45" s="8" t="s">
-        <v>134</v>
+        <v>22</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>46</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="H45" s="5"/>
       <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" ht="67.2" thickBot="1">
       <c r="A46" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>184</v>
+        <v>139</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="D46" s="5"/>
-      <c r="E46" s="8">
+        <v>161</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H46" s="5"/>
+      <c r="I46" s="1"/>
+    </row>
+    <row r="47" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A47" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E47" s="8">
         <v>123456789</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="I46" s="1"/>
-    </row>
-    <row r="47" spans="1:9" ht="54" thickBot="1">
-      <c r="A47" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D47" s="5"/>
-      <c r="E47" s="8" t="s">
-        <v>53</v>
-      </c>
       <c r="F47" s="1" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>182</v>
-      </c>
+        <v>279</v>
+      </c>
+      <c r="H47" s="5"/>
       <c r="I47" s="1"/>
     </row>
     <row r="48" spans="1:9" ht="54" thickBot="1">
       <c r="A48" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D48" s="5"/>
+        <v>157</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E48" s="8" t="s">
-        <v>174</v>
+        <v>53</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>183</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="H48" s="5"/>
       <c r="I48" s="1"/>
     </row>
     <row r="49" spans="1:9" ht="54" thickBot="1">
       <c r="A49" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="D49" s="5"/>
+        <v>158</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E49" s="8" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>183</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="H49" s="5"/>
       <c r="I49" s="1"/>
     </row>
     <row r="50" spans="1:9" ht="54" thickBot="1">
       <c r="A50" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="D50" s="5"/>
+        <v>159</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>260</v>
+      </c>
       <c r="E50" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G50" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>46</v>
-      </c>
+      <c r="H50" s="5"/>
       <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" ht="54" thickBot="1">
       <c r="A51" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="D51" s="5"/>
-      <c r="E51" s="10" t="s">
-        <v>188</v>
+        <v>160</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>170</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>179</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="H51" s="5"/>
+      <c r="I51" s="1"/>
     </row>
     <row r="52" spans="1:9" ht="54" thickBot="1">
       <c r="A52" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B52" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D52" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="H52" s="5"/>
+      <c r="I52" s="1"/>
+    </row>
+    <row r="53" spans="1:9" ht="54" thickBot="1">
+      <c r="A53" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D53" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="H53" s="5"/>
+      <c r="I53" s="1"/>
+    </row>
+    <row r="54" spans="1:9" ht="54" thickBot="1">
+      <c r="A54" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H54" s="5"/>
+      <c r="I54" s="1"/>
+    </row>
+    <row r="55" spans="1:9" ht="54" thickBot="1">
+      <c r="A55" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H55" s="5"/>
+      <c r="I55" s="1"/>
+    </row>
+    <row r="56" spans="1:9" ht="54" thickBot="1">
+      <c r="A56" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H56" s="5"/>
+      <c r="I56" s="1"/>
+    </row>
+    <row r="57" spans="1:9" ht="54" thickBot="1">
+      <c r="A57" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B57" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C57" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="H57" s="5"/>
+      <c r="I57" s="1"/>
+    </row>
+    <row r="58" spans="1:9" ht="54" thickBot="1">
+      <c r="A58" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B58" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="D52" s="5"/>
-      <c r="E52" s="10" t="s">
+      <c r="C58" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E58" s="8">
+        <v>123456789</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="H58" s="5"/>
+      <c r="I58" s="1"/>
+    </row>
+    <row r="59" spans="1:9" ht="54" thickBot="1">
+      <c r="A59" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B59" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="F52" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" ht="15" thickBot="1">
-      <c r="A53" s="5"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="8"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="4"/>
-    </row>
-    <row r="54" spans="1:9" ht="15" thickBot="1">
-      <c r="A54" s="5"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="8"/>
-      <c r="F54" s="1"/>
-      <c r="G54" s="4"/>
-    </row>
-    <row r="55" spans="1:9" ht="15" thickBot="1">
-      <c r="A55" s="5"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="8"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="4"/>
-    </row>
-    <row r="56" spans="1:9" ht="15" thickBot="1">
-      <c r="A56" s="5"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="4"/>
-    </row>
-    <row r="57" spans="1:9" ht="15" thickBot="1">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="8"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="4"/>
-    </row>
-    <row r="58" spans="1:9" ht="15" thickBot="1">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="8"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="4"/>
-    </row>
-    <row r="59" spans="1:9" ht="15" thickBot="1">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="4"/>
-    </row>
-    <row r="60" spans="1:9" ht="15" thickBot="1">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="4"/>
-    </row>
-    <row r="61" spans="1:9" ht="15" thickBot="1">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="8"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="4"/>
-    </row>
-    <row r="62" spans="1:9" ht="15" thickBot="1">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="8"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="4"/>
-    </row>
-    <row r="63" spans="1:9" ht="15" thickBot="1">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="8"/>
-      <c r="F63" s="1"/>
-      <c r="G63" s="4"/>
-    </row>
-    <row r="64" spans="1:9" ht="15" thickBot="1">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="1"/>
-      <c r="G64" s="4"/>
-    </row>
-    <row r="65" spans="1:7" ht="15" thickBot="1">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="8"/>
-      <c r="F65" s="1"/>
-      <c r="G65" s="4"/>
-    </row>
-    <row r="66" spans="1:7" ht="15" thickBot="1">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="8"/>
-      <c r="F66" s="1"/>
-      <c r="G66" s="4"/>
-    </row>
-    <row r="67" spans="1:7" ht="15" thickBot="1">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="1"/>
-      <c r="G67" s="4"/>
-    </row>
-    <row r="68" spans="1:7" ht="15" thickBot="1">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="8"/>
-      <c r="F68" s="1"/>
-      <c r="G68" s="4"/>
-    </row>
-    <row r="69" spans="1:7" ht="15" thickBot="1">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="8"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="4"/>
-    </row>
-    <row r="70" spans="1:7" ht="15" thickBot="1">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="8"/>
-      <c r="F70" s="1"/>
-      <c r="G70" s="4"/>
-    </row>
-    <row r="71" spans="1:7" ht="15" thickBot="1">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="8"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="4"/>
-    </row>
-    <row r="72" spans="1:7" ht="15" thickBot="1">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="8"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="4"/>
-    </row>
-    <row r="73" spans="1:7" ht="15" thickBot="1">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="8"/>
-      <c r="F73" s="1"/>
-      <c r="G73" s="4"/>
-    </row>
-    <row r="74" spans="1:7" ht="15" thickBot="1">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="8"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="4"/>
-    </row>
-    <row r="75" spans="1:7" ht="15" thickBot="1">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="8"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="4"/>
-    </row>
-    <row r="76" spans="1:7" ht="15" thickBot="1">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="8"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="4"/>
-    </row>
-    <row r="77" spans="1:7" ht="15" thickBot="1">
-      <c r="A77" s="5"/>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="8"/>
-      <c r="F77" s="1"/>
-      <c r="G77" s="4"/>
-    </row>
-    <row r="78" spans="1:7" ht="15" thickBot="1">
-      <c r="A78" s="5"/>
-      <c r="B78" s="5"/>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="8"/>
-      <c r="F78" s="1"/>
-      <c r="G78" s="4"/>
-    </row>
-    <row r="79" spans="1:7" ht="15" thickBot="1">
-      <c r="A79" s="5"/>
-      <c r="B79" s="5"/>
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="1"/>
-      <c r="G79" s="4"/>
-    </row>
-    <row r="80" spans="1:7" ht="15" thickBot="1">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="8"/>
-      <c r="F80" s="1"/>
-      <c r="G80" s="4"/>
-    </row>
-    <row r="81" spans="1:6" ht="15" thickBot="1">
+      <c r="C59" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H59" s="5"/>
+      <c r="I59" s="1"/>
+    </row>
+    <row r="60" spans="1:9" ht="54" thickBot="1">
+      <c r="A60" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H60" s="5"/>
+      <c r="I60" s="1"/>
+    </row>
+    <row r="61" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A61" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="H61" s="5"/>
+      <c r="I61" s="1"/>
+    </row>
+    <row r="62" spans="1:9" ht="54" thickBot="1">
+      <c r="A62" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D62" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="H62" s="5"/>
+      <c r="I62" s="1"/>
+    </row>
+    <row r="63" spans="1:9" ht="54" thickBot="1">
+      <c r="A63" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D63" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E63" s="8">
+        <v>123456789</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="H63" s="5"/>
+      <c r="I63" s="1"/>
+    </row>
+    <row r="64" spans="1:9" ht="54" thickBot="1">
+      <c r="A64" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H64" s="5"/>
+      <c r="I64" s="1"/>
+    </row>
+    <row r="65" spans="1:9" ht="54" thickBot="1">
+      <c r="A65" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E65" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H65" s="5"/>
+      <c r="I65" s="1"/>
+    </row>
+    <row r="66" spans="1:9" ht="54" thickBot="1">
+      <c r="A66" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="H66" s="5"/>
+      <c r="I66" s="1"/>
+    </row>
+    <row r="67" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A67" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E67" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H67" s="5"/>
+      <c r="I67" s="1"/>
+    </row>
+    <row r="68" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A68" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E68" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H68" s="5"/>
+      <c r="I68" s="1"/>
+    </row>
+    <row r="69" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A69" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E69" s="8">
+        <v>0</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="H69" s="5"/>
+      <c r="I69" s="1"/>
+    </row>
+    <row r="70" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A70" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E70" s="8">
+        <v>-1</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G70" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="H70" s="5"/>
+      <c r="I70" s="1"/>
+    </row>
+    <row r="71" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A71" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E71" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="H71" s="5"/>
+      <c r="I71" s="1"/>
+    </row>
+    <row r="72" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A72" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D72" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E72" s="8">
+        <v>1</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="H72" s="5"/>
+      <c r="I72" s="1"/>
+    </row>
+    <row r="73" spans="1:9" ht="54" thickBot="1">
+      <c r="A73" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D73" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="H73" s="5"/>
+      <c r="I73" s="1"/>
+    </row>
+    <row r="74" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A74" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G74" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="H74" s="5"/>
+      <c r="I74" s="1"/>
+    </row>
+    <row r="75" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A75" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D75" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H75" s="5"/>
+      <c r="I75" s="1"/>
+    </row>
+    <row r="76" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A76" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="D76" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E76" s="8">
+        <v>1</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="H76" s="5"/>
+      <c r="I76" s="1"/>
+    </row>
+    <row r="77" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A77" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D77" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E77" s="8">
+        <v>-1</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="H77" s="5"/>
+      <c r="I77" s="1"/>
+    </row>
+    <row r="78" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A78" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D78" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E78" s="8">
+        <v>1E-4</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G78" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="H78" s="5"/>
+      <c r="I78" s="1"/>
+    </row>
+    <row r="79" spans="1:9" ht="67.2" thickBot="1">
+      <c r="A79" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="D79" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E79" s="8">
+        <v>0</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G79" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="H79" s="5"/>
+      <c r="I79" s="1"/>
+    </row>
+    <row r="80" spans="1:9" ht="83.4" thickBot="1">
+      <c r="A80" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B80" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="C80" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D80" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E80" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="G80" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="H80" s="5"/>
+      <c r="I80" s="1"/>
+    </row>
+    <row r="81" spans="1:9" ht="15" thickBot="1">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
+      <c r="D81" s="12"/>
       <c r="E81" s="8"/>
       <c r="F81" s="1"/>
-    </row>
-    <row r="82" spans="1:6" ht="15" thickBot="1">
+      <c r="G81" s="4"/>
+      <c r="H81" s="5"/>
+      <c r="I81" s="1"/>
+    </row>
+    <row r="82" spans="1:9" ht="15" thickBot="1">
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
       <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
+      <c r="D82" s="12"/>
       <c r="E82" s="8"/>
       <c r="F82" s="1"/>
-    </row>
-    <row r="83" spans="1:6" ht="15" thickBot="1">
+      <c r="G82" s="4"/>
+      <c r="H82" s="5"/>
+      <c r="I82" s="1"/>
+    </row>
+    <row r="83" spans="1:9" ht="15" thickBot="1">
       <c r="A83" s="5"/>
       <c r="B83" s="5"/>
       <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
+      <c r="D83" s="12"/>
       <c r="E83" s="8"/>
       <c r="F83" s="1"/>
-    </row>
-    <row r="84" spans="1:6" ht="15" thickBot="1">
+      <c r="G83" s="4"/>
+      <c r="H83" s="5"/>
+      <c r="I83" s="1"/>
+    </row>
+    <row r="84" spans="1:9" ht="15" thickBot="1">
       <c r="A84" s="5"/>
       <c r="B84" s="5"/>
       <c r="C84" s="5"/>
-      <c r="D84" s="5"/>
+      <c r="D84" s="12"/>
       <c r="E84" s="8"/>
       <c r="F84" s="1"/>
-    </row>
-    <row r="85" spans="1:6" ht="15" thickBot="1">
+      <c r="G84" s="4"/>
+      <c r="H84" s="5"/>
+      <c r="I84" s="1"/>
+    </row>
+    <row r="85" spans="1:9" ht="15" thickBot="1">
       <c r="A85" s="5"/>
       <c r="B85" s="5"/>
       <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
+      <c r="D85" s="12"/>
       <c r="E85" s="8"/>
       <c r="F85" s="1"/>
-    </row>
-    <row r="86" spans="1:6" ht="15" thickBot="1">
+      <c r="G85" s="4"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="1"/>
+    </row>
+    <row r="86" spans="1:9" ht="15" thickBot="1">
       <c r="A86" s="5"/>
       <c r="B86" s="5"/>
       <c r="C86" s="5"/>
-      <c r="D86" s="5"/>
+      <c r="D86" s="12"/>
       <c r="E86" s="8"/>
       <c r="F86" s="1"/>
-    </row>
-    <row r="87" spans="1:6" ht="15" thickBot="1">
+      <c r="G86" s="4"/>
+      <c r="H86" s="5"/>
+      <c r="I86" s="1"/>
+    </row>
+    <row r="87" spans="1:9" ht="15" thickBot="1">
       <c r="A87" s="5"/>
       <c r="B87" s="5"/>
       <c r="C87" s="5"/>
-      <c r="D87" s="5"/>
+      <c r="D87" s="12"/>
       <c r="E87" s="8"/>
       <c r="F87" s="1"/>
-    </row>
-    <row r="88" spans="1:6" ht="15" thickBot="1">
+      <c r="G87" s="4"/>
+      <c r="H87" s="5"/>
+      <c r="I87" s="1"/>
+    </row>
+    <row r="88" spans="1:9" ht="15" thickBot="1">
       <c r="A88" s="5"/>
       <c r="B88" s="5"/>
       <c r="C88" s="5"/>
-      <c r="D88" s="5"/>
+      <c r="D88" s="12"/>
       <c r="E88" s="8"/>
       <c r="F88" s="1"/>
-    </row>
-    <row r="89" spans="1:6" ht="15" thickBot="1">
+      <c r="G88" s="4"/>
+      <c r="H88" s="5"/>
+      <c r="I88" s="1"/>
+    </row>
+    <row r="89" spans="1:9" ht="15" thickBot="1">
       <c r="A89" s="5"/>
       <c r="B89" s="5"/>
       <c r="C89" s="5"/>
-      <c r="D89" s="5"/>
+      <c r="D89" s="12"/>
       <c r="E89" s="8"/>
       <c r="F89" s="1"/>
-    </row>
-    <row r="90" spans="1:6" ht="15" thickBot="1">
+      <c r="G89" s="4"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="1"/>
+    </row>
+    <row r="90" spans="1:9" ht="15" thickBot="1">
       <c r="A90" s="5"/>
       <c r="B90" s="5"/>
       <c r="C90" s="5"/>
-      <c r="D90" s="5"/>
+      <c r="D90" s="12"/>
       <c r="E90" s="8"/>
       <c r="F90" s="1"/>
-    </row>
-    <row r="91" spans="1:6" ht="15" thickBot="1">
+      <c r="G90" s="4"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="1"/>
+    </row>
+    <row r="91" spans="1:9" ht="15" thickBot="1">
       <c r="A91" s="5"/>
       <c r="B91" s="5"/>
       <c r="C91" s="5"/>
-      <c r="D91" s="5"/>
+      <c r="D91" s="12"/>
       <c r="E91" s="8"/>
       <c r="F91" s="1"/>
-    </row>
-    <row r="92" spans="1:6" ht="15" thickBot="1">
+      <c r="G91" s="4"/>
+      <c r="H91" s="5"/>
+      <c r="I91" s="1"/>
+    </row>
+    <row r="92" spans="1:9" ht="15" thickBot="1">
       <c r="A92" s="5"/>
       <c r="B92" s="5"/>
       <c r="C92" s="5"/>
-      <c r="D92" s="5"/>
+      <c r="D92" s="12"/>
       <c r="E92" s="8"/>
       <c r="F92" s="1"/>
-    </row>
-    <row r="93" spans="1:6" ht="15" thickBot="1">
+      <c r="G92" s="4"/>
+      <c r="H92" s="5"/>
+      <c r="I92" s="1"/>
+    </row>
+    <row r="93" spans="1:9" ht="15" thickBot="1">
       <c r="A93" s="5"/>
       <c r="B93" s="5"/>
       <c r="C93" s="5"/>
-      <c r="D93" s="5"/>
+      <c r="D93" s="12"/>
       <c r="E93" s="8"/>
       <c r="F93" s="1"/>
-    </row>
-    <row r="94" spans="1:6" ht="15" thickBot="1">
+      <c r="G93" s="4"/>
+      <c r="H93" s="5"/>
+      <c r="I93" s="1"/>
+    </row>
+    <row r="94" spans="1:9" ht="15" thickBot="1">
       <c r="A94" s="5"/>
       <c r="B94" s="5"/>
       <c r="C94" s="5"/>
-      <c r="D94" s="5"/>
+      <c r="D94" s="12"/>
       <c r="E94" s="8"/>
       <c r="F94" s="1"/>
-    </row>
-    <row r="95" spans="1:6" ht="15" thickBot="1">
+      <c r="G94" s="4"/>
+      <c r="H94" s="5"/>
+      <c r="I94" s="1"/>
+    </row>
+    <row r="95" spans="1:9" ht="15" thickBot="1">
       <c r="A95" s="5"/>
       <c r="B95" s="5"/>
       <c r="C95" s="5"/>
-      <c r="D95" s="5"/>
+      <c r="D95" s="12"/>
       <c r="E95" s="8"/>
       <c r="F95" s="1"/>
-    </row>
-    <row r="96" spans="1:6" ht="15" thickBot="1">
+      <c r="G95" s="4"/>
+      <c r="H95" s="5"/>
+      <c r="I95" s="1"/>
+    </row>
+    <row r="96" spans="1:9" ht="15" thickBot="1">
       <c r="A96" s="5"/>
       <c r="B96" s="5"/>
       <c r="C96" s="5"/>
-      <c r="D96" s="5"/>
+      <c r="D96" s="12"/>
       <c r="E96" s="8"/>
       <c r="F96" s="1"/>
-    </row>
-    <row r="97" spans="1:6" ht="15" thickBot="1">
+      <c r="G96" s="4"/>
+      <c r="H96" s="5"/>
+      <c r="I96" s="1"/>
+    </row>
+    <row r="97" spans="1:9" ht="15" thickBot="1">
       <c r="A97" s="5"/>
       <c r="B97" s="5"/>
       <c r="C97" s="5"/>
-      <c r="D97" s="5"/>
+      <c r="D97" s="12"/>
       <c r="E97" s="8"/>
       <c r="F97" s="1"/>
-    </row>
-    <row r="98" spans="1:6" ht="15" thickBot="1">
+      <c r="G97" s="4"/>
+      <c r="H97" s="5"/>
+      <c r="I97" s="1"/>
+    </row>
+    <row r="98" spans="1:9" ht="15" thickBot="1">
       <c r="A98" s="5"/>
       <c r="B98" s="5"/>
       <c r="C98" s="5"/>
-      <c r="D98" s="5"/>
+      <c r="D98" s="12"/>
       <c r="E98" s="8"/>
       <c r="F98" s="1"/>
-    </row>
-    <row r="99" spans="1:6" ht="15" thickBot="1">
+      <c r="G98" s="4"/>
+      <c r="H98" s="5"/>
+      <c r="I98" s="1"/>
+    </row>
+    <row r="99" spans="1:9" ht="15" thickBot="1">
       <c r="A99" s="5"/>
       <c r="B99" s="5"/>
       <c r="C99" s="5"/>
-      <c r="D99" s="5"/>
+      <c r="D99" s="12"/>
       <c r="E99" s="8"/>
       <c r="F99" s="1"/>
-    </row>
-    <row r="100" spans="1:6" ht="15" thickBot="1">
+      <c r="G99" s="4"/>
+      <c r="H99" s="5"/>
+      <c r="I99" s="1"/>
+    </row>
+    <row r="100" spans="1:9" ht="15" thickBot="1">
       <c r="A100" s="5"/>
       <c r="B100" s="5"/>
       <c r="C100" s="5"/>
-      <c r="D100" s="5"/>
+      <c r="D100" s="12"/>
       <c r="E100" s="8"/>
       <c r="F100" s="1"/>
-    </row>
-    <row r="101" spans="1:6" ht="15" thickBot="1">
+      <c r="G100" s="4"/>
+      <c r="H100" s="5"/>
+      <c r="I100" s="1"/>
+    </row>
+    <row r="101" spans="1:9" ht="15" thickBot="1">
       <c r="A101" s="5"/>
       <c r="B101" s="5"/>
       <c r="C101" s="5"/>
-      <c r="D101" s="5"/>
+      <c r="D101" s="12"/>
       <c r="E101" s="8"/>
       <c r="F101" s="1"/>
-    </row>
-    <row r="102" spans="1:6" ht="15" thickBot="1">
+      <c r="G101" s="4"/>
+      <c r="H101" s="5"/>
+      <c r="I101" s="1"/>
+    </row>
+    <row r="102" spans="1:9" ht="15" thickBot="1">
       <c r="A102" s="5"/>
       <c r="B102" s="5"/>
       <c r="C102" s="5"/>
-      <c r="D102" s="5"/>
+      <c r="D102" s="12"/>
       <c r="E102" s="8"/>
       <c r="F102" s="1"/>
-    </row>
-    <row r="103" spans="1:6" ht="15" thickBot="1">
+      <c r="G102" s="4"/>
+      <c r="H102" s="5"/>
+      <c r="I102" s="1"/>
+    </row>
+    <row r="103" spans="1:9" ht="15" thickBot="1">
       <c r="A103" s="5"/>
+      <c r="B103" s="5"/>
       <c r="C103" s="5"/>
-      <c r="D103" s="5"/>
+      <c r="D103" s="12"/>
       <c r="E103" s="8"/>
       <c r="F103" s="1"/>
-    </row>
-    <row r="104" spans="1:6" ht="15" thickBot="1">
+      <c r="G103" s="4"/>
+      <c r="H103" s="5"/>
+      <c r="I103" s="1"/>
+    </row>
+    <row r="104" spans="1:9" ht="15" thickBot="1">
       <c r="A104" s="5"/>
+      <c r="B104" s="5"/>
+      <c r="C104" s="5"/>
+      <c r="D104" s="12"/>
       <c r="E104" s="8"/>
       <c r="F104" s="1"/>
-    </row>
-    <row r="105" spans="1:6" ht="15" thickBot="1">
+      <c r="G104" s="4"/>
+      <c r="H104" s="5"/>
+      <c r="I104" s="1"/>
+    </row>
+    <row r="105" spans="1:9" ht="15" thickBot="1">
       <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
+      <c r="C105" s="5"/>
+      <c r="D105" s="12"/>
       <c r="E105" s="8"/>
       <c r="F105" s="1"/>
-    </row>
-    <row r="106" spans="1:6" ht="15" thickBot="1">
+      <c r="G105" s="4"/>
+      <c r="H105" s="5"/>
+      <c r="I105" s="1"/>
+    </row>
+    <row r="106" spans="1:9" ht="15" thickBot="1">
       <c r="A106" s="5"/>
+      <c r="B106" s="5"/>
+      <c r="C106" s="5"/>
+      <c r="D106" s="12"/>
+      <c r="E106" s="8"/>
       <c r="F106" s="1"/>
-    </row>
-    <row r="107" spans="1:6" ht="15" thickBot="1">
+      <c r="G106" s="4"/>
+      <c r="H106" s="5"/>
+      <c r="I106" s="1"/>
+    </row>
+    <row r="107" spans="1:9" ht="15" thickBot="1">
       <c r="A107" s="5"/>
+      <c r="B107" s="5"/>
+      <c r="C107" s="5"/>
+      <c r="D107" s="12"/>
+      <c r="E107" s="8"/>
       <c r="F107" s="1"/>
-    </row>
-    <row r="108" spans="1:6" ht="15" thickBot="1">
+      <c r="G107" s="4"/>
+      <c r="H107" s="5"/>
+      <c r="I107" s="1"/>
+    </row>
+    <row r="108" spans="1:9" ht="15" thickBot="1">
       <c r="A108" s="5"/>
-    </row>
-    <row r="109" spans="1:6" ht="15" thickBot="1">
+      <c r="B108" s="5"/>
+      <c r="C108" s="5"/>
+      <c r="D108" s="12"/>
+      <c r="E108" s="8"/>
+      <c r="F108" s="1"/>
+      <c r="G108" s="4"/>
+      <c r="H108" s="5"/>
+      <c r="I108" s="1"/>
+    </row>
+    <row r="109" spans="1:9" ht="15" thickBot="1">
       <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
+      <c r="C109" s="5"/>
+      <c r="D109" s="12"/>
+      <c r="E109" s="8"/>
+      <c r="F109" s="1"/>
+      <c r="G109" s="4"/>
+      <c r="H109" s="5"/>
+      <c r="I109" s="1"/>
+    </row>
+    <row r="110" spans="1:9" ht="15" thickBot="1">
+      <c r="A110" s="5"/>
+      <c r="B110" s="5"/>
+      <c r="C110" s="5"/>
+      <c r="D110" s="12"/>
+      <c r="E110" s="8"/>
+      <c r="F110" s="1"/>
+      <c r="G110" s="4"/>
+      <c r="H110" s="5"/>
+      <c r="I110" s="1"/>
+    </row>
+    <row r="111" spans="1:9" ht="15" thickBot="1">
+      <c r="A111" s="5"/>
+      <c r="B111" s="5"/>
+      <c r="C111" s="5"/>
+      <c r="D111" s="12"/>
+      <c r="E111" s="8"/>
+      <c r="F111" s="1"/>
+      <c r="G111" s="4"/>
+      <c r="H111" s="5"/>
+      <c r="I111" s="1"/>
+    </row>
+    <row r="112" spans="1:9" ht="15" thickBot="1">
+      <c r="A112" s="5"/>
+      <c r="B112" s="5"/>
+      <c r="C112" s="5"/>
+      <c r="D112" s="12"/>
+      <c r="E112" s="8"/>
+      <c r="F112" s="1"/>
+      <c r="G112" s="4"/>
+      <c r="H112" s="5"/>
+      <c r="I112" s="1"/>
+    </row>
+    <row r="113" spans="1:9" ht="15" thickBot="1">
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
+      <c r="C113" s="5"/>
+      <c r="D113" s="12"/>
+      <c r="E113" s="8"/>
+      <c r="F113" s="1"/>
+      <c r="G113" s="4"/>
+      <c r="H113" s="5"/>
+      <c r="I113" s="1"/>
+    </row>
+    <row r="114" spans="1:9" ht="15" thickBot="1">
+      <c r="A114" s="5"/>
+      <c r="B114" s="5"/>
+      <c r="C114" s="5"/>
+      <c r="D114" s="12"/>
+      <c r="E114" s="8"/>
+      <c r="F114" s="1"/>
+      <c r="G114" s="4"/>
+      <c r="H114" s="5"/>
+      <c r="I114" s="1"/>
+    </row>
+    <row r="115" spans="1:9" ht="15" thickBot="1">
+      <c r="A115" s="5"/>
+      <c r="B115" s="5"/>
+      <c r="C115" s="5"/>
+      <c r="D115" s="12"/>
+      <c r="E115" s="8"/>
+      <c r="F115" s="1"/>
+      <c r="G115" s="4"/>
+      <c r="H115" s="5"/>
+      <c r="I115" s="1"/>
+    </row>
+    <row r="116" spans="1:9" ht="15" thickBot="1">
+      <c r="A116" s="5"/>
+      <c r="B116" s="5"/>
+      <c r="C116" s="5"/>
+      <c r="D116" s="12"/>
+      <c r="E116" s="8"/>
+      <c r="G116" s="4"/>
+      <c r="H116" s="5"/>
+      <c r="I116" s="1"/>
+    </row>
+    <row r="117" spans="1:9" ht="15" thickBot="1">
+      <c r="H117" s="5"/>
+      <c r="I117" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E49" r:id="rId1" xr:uid="{22256702-EAD2-4D11-BAAB-31B3929E3CDF}"/>
-    <hyperlink ref="E51" r:id="rId2" display="Test@test.com" xr:uid="{1E184A82-84D9-406A-9A4D-713909ABFAE9}"/>
-    <hyperlink ref="E52" r:id="rId3" xr:uid="{46418758-D47A-46EE-8F73-62CD45A95A9A}"/>
+    <hyperlink ref="E50" r:id="rId1" xr:uid="{22256702-EAD2-4D11-BAAB-31B3929E3CDF}"/>
+    <hyperlink ref="E52" r:id="rId2" display="Test@test.com" xr:uid="{1E184A82-84D9-406A-9A4D-713909ABFAE9}"/>
+    <hyperlink ref="E53" r:id="rId3" xr:uid="{46418758-D47A-46EE-8F73-62CD45A95A9A}"/>
+    <hyperlink ref="E60" r:id="rId4" xr:uid="{8DFE2CA8-F230-430B-9E32-9AA6FBACBCC1}"/>
+    <hyperlink ref="E67" r:id="rId5" xr:uid="{624B3634-8D40-4E0D-A10E-D96DF9FBCC88}"/>
+    <hyperlink ref="E75" r:id="rId6" xr:uid="{6DC6E8F3-3EAF-4F2A-9856-2AAFB96321EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>